<commit_message>
Use fresh saved match pages for dataset build
</commit_message>
<xml_diff>
--- a/data/tournaments_master.xlsx
+++ b/data/tournaments_master.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3189,7 +3189,7 @@
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5289,7 +5289,7 @@
       </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5541,7 +5541,7 @@
       </c>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5793,7 +5793,7 @@
       </c>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -6213,7 +6213,7 @@
       </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -6381,7 +6381,7 @@
       </c>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6717,7 +6717,7 @@
       </c>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -7053,7 +7053,7 @@
       </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -7137,7 +7137,7 @@
       </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -7221,7 +7221,7 @@
       </c>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -7305,7 +7305,7 @@
       </c>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
       </c>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -7557,7 +7557,7 @@
       </c>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -7641,7 +7641,7 @@
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
       </c>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -7893,7 +7893,7 @@
       </c>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -7977,7 +7977,7 @@
       </c>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
       </c>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -8313,7 +8313,7 @@
       </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -8397,7 +8397,7 @@
       </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -8481,7 +8481,7 @@
       </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -8565,7 +8565,7 @@
       </c>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -8733,7 +8733,7 @@
       </c>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
       </c>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -9069,7 +9069,7 @@
       </c>
       <c r="M103" t="inlineStr"/>
       <c r="N103" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -9153,7 +9153,7 @@
       </c>
       <c r="M104" t="inlineStr"/>
       <c r="N104" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -9237,7 +9237,7 @@
       </c>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -9321,7 +9321,7 @@
       </c>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -9573,7 +9573,7 @@
       </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -9657,7 +9657,7 @@
       </c>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -9909,7 +9909,7 @@
       </c>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -9993,7 +9993,7 @@
       </c>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -10077,7 +10077,7 @@
       </c>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -10161,7 +10161,7 @@
       </c>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
       </c>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -10329,7 +10329,7 @@
       </c>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -10413,7 +10413,7 @@
       </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -10497,7 +10497,7 @@
       </c>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
       </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -10665,7 +10665,7 @@
       </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -10917,7 +10917,7 @@
       </c>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O125" t="inlineStr">
         <is>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -11085,7 +11085,7 @@
       </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -11169,7 +11169,7 @@
       </c>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -11337,7 +11337,7 @@
       </c>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -11505,7 +11505,7 @@
       </c>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -11673,7 +11673,7 @@
       </c>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -11757,7 +11757,7 @@
       </c>
       <c r="M135" t="inlineStr"/>
       <c r="N135" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -11841,7 +11841,7 @@
       </c>
       <c r="M136" t="inlineStr"/>
       <c r="N136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -11925,7 +11925,7 @@
       </c>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -12009,7 +12009,7 @@
       </c>
       <c r="M138" t="inlineStr"/>
       <c r="N138" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -12093,7 +12093,7 @@
       </c>
       <c r="M139" t="inlineStr"/>
       <c r="N139" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -12177,7 +12177,7 @@
       </c>
       <c r="M140" t="inlineStr"/>
       <c r="N140" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -12261,7 +12261,7 @@
       </c>
       <c r="M141" t="inlineStr"/>
       <c r="N141" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -12345,7 +12345,7 @@
       </c>
       <c r="M142" t="inlineStr"/>
       <c r="N142" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="M143" t="inlineStr"/>
       <c r="N143" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -12513,7 +12513,7 @@
       </c>
       <c r="M144" t="inlineStr"/>
       <c r="N144" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -12681,7 +12681,7 @@
       </c>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -12765,7 +12765,7 @@
       </c>
       <c r="M147" t="inlineStr"/>
       <c r="N147" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -12849,7 +12849,7 @@
       </c>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -12933,7 +12933,7 @@
       </c>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
       </c>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -13101,7 +13101,7 @@
       </c>
       <c r="M151" t="inlineStr"/>
       <c r="N151" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -13185,7 +13185,7 @@
       </c>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -13269,7 +13269,7 @@
       </c>
       <c r="M153" t="inlineStr"/>
       <c r="N153" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -13353,7 +13353,7 @@
       </c>
       <c r="M154" t="inlineStr"/>
       <c r="N154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -13437,7 +13437,7 @@
       </c>
       <c r="M155" t="inlineStr"/>
       <c r="N155" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -13521,7 +13521,7 @@
       </c>
       <c r="M156" t="inlineStr"/>
       <c r="N156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -13605,7 +13605,7 @@
       </c>
       <c r="M157" t="inlineStr"/>
       <c r="N157" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
@@ -13689,7 +13689,7 @@
       </c>
       <c r="M158" t="inlineStr"/>
       <c r="N158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O158" t="inlineStr">
         <is>
@@ -13773,7 +13773,7 @@
       </c>
       <c r="M159" t="inlineStr"/>
       <c r="N159" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -13857,7 +13857,7 @@
       </c>
       <c r="M160" t="inlineStr"/>
       <c r="N160" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
@@ -13941,7 +13941,7 @@
       </c>
       <c r="M161" t="inlineStr"/>
       <c r="N161" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -14025,7 +14025,7 @@
       </c>
       <c r="M162" t="inlineStr"/>
       <c r="N162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -14109,7 +14109,7 @@
       </c>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -14193,7 +14193,7 @@
       </c>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
@@ -14277,7 +14277,7 @@
       </c>
       <c r="M165" t="inlineStr"/>
       <c r="N165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -14361,7 +14361,7 @@
       </c>
       <c r="M166" t="inlineStr"/>
       <c r="N166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
@@ -14445,7 +14445,7 @@
       </c>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O167" t="inlineStr">
         <is>
@@ -14529,7 +14529,7 @@
       </c>
       <c r="M168" t="inlineStr"/>
       <c r="N168" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O168" t="inlineStr">
         <is>
@@ -14613,7 +14613,7 @@
       </c>
       <c r="M169" t="inlineStr"/>
       <c r="N169" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
@@ -14697,7 +14697,7 @@
       </c>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O170" t="inlineStr">
         <is>
@@ -14781,7 +14781,7 @@
       </c>
       <c r="M171" t="inlineStr"/>
       <c r="N171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -14865,7 +14865,7 @@
       </c>
       <c r="M172" t="inlineStr"/>
       <c r="N172" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
@@ -14949,7 +14949,7 @@
       </c>
       <c r="M173" t="inlineStr"/>
       <c r="N173" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O173" t="inlineStr">
         <is>
@@ -15033,7 +15033,7 @@
       </c>
       <c r="M174" t="inlineStr"/>
       <c r="N174" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -15117,7 +15117,7 @@
       </c>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -15201,7 +15201,7 @@
       </c>
       <c r="M176" t="inlineStr"/>
       <c r="N176" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
@@ -15285,7 +15285,7 @@
       </c>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
@@ -15369,7 +15369,7 @@
       </c>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
@@ -15453,7 +15453,7 @@
       </c>
       <c r="M179" t="inlineStr"/>
       <c r="N179" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O179" t="inlineStr">
         <is>
@@ -15537,7 +15537,7 @@
       </c>
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O180" t="inlineStr">
         <is>
@@ -15621,7 +15621,7 @@
       </c>
       <c r="M181" t="inlineStr"/>
       <c r="N181" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
@@ -15705,7 +15705,7 @@
       </c>
       <c r="M182" t="inlineStr"/>
       <c r="N182" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
@@ -15789,7 +15789,7 @@
       </c>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -15873,7 +15873,7 @@
       </c>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -15957,7 +15957,7 @@
       </c>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -16041,7 +16041,7 @@
       </c>
       <c r="M186" t="inlineStr"/>
       <c r="N186" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O186" t="inlineStr">
         <is>
@@ -16125,7 +16125,7 @@
       </c>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O187" t="inlineStr">
         <is>
@@ -16209,7 +16209,7 @@
       </c>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -16293,7 +16293,7 @@
       </c>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O189" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
       </c>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -16461,7 +16461,7 @@
       </c>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O191" t="inlineStr">
         <is>
@@ -16545,7 +16545,7 @@
       </c>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O192" t="inlineStr">
         <is>
@@ -16629,7 +16629,7 @@
       </c>
       <c r="M193" t="inlineStr"/>
       <c r="N193" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -16713,7 +16713,7 @@
       </c>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -16881,7 +16881,7 @@
       </c>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -16965,7 +16965,7 @@
       </c>
       <c r="M197" t="inlineStr"/>
       <c r="N197" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O197" t="inlineStr">
         <is>
@@ -17049,7 +17049,7 @@
       </c>
       <c r="M198" t="inlineStr"/>
       <c r="N198" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O198" t="inlineStr">
         <is>
@@ -17133,7 +17133,7 @@
       </c>
       <c r="M199" t="inlineStr"/>
       <c r="N199" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -17217,7 +17217,7 @@
       </c>
       <c r="M200" t="inlineStr"/>
       <c r="N200" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -17301,7 +17301,7 @@
       </c>
       <c r="M201" t="inlineStr"/>
       <c r="N201" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O201" t="inlineStr">
         <is>
@@ -17385,7 +17385,7 @@
       </c>
       <c r="M202" t="inlineStr"/>
       <c r="N202" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O202" t="inlineStr">
         <is>
@@ -17469,7 +17469,7 @@
       </c>
       <c r="M203" t="inlineStr"/>
       <c r="N203" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O203" t="inlineStr">
         <is>
@@ -17553,7 +17553,7 @@
       </c>
       <c r="M204" t="inlineStr"/>
       <c r="N204" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O204" t="inlineStr">
         <is>
@@ -17637,7 +17637,7 @@
       </c>
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -17721,7 +17721,7 @@
       </c>
       <c r="M206" t="inlineStr"/>
       <c r="N206" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -17805,7 +17805,7 @@
       </c>
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O207" t="inlineStr">
         <is>
@@ -17889,7 +17889,7 @@
       </c>
       <c r="M208" t="inlineStr"/>
       <c r="N208" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -17973,7 +17973,7 @@
       </c>
       <c r="M209" t="inlineStr"/>
       <c r="N209" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O209" t="inlineStr">
         <is>
@@ -18057,7 +18057,7 @@
       </c>
       <c r="M210" t="inlineStr"/>
       <c r="N210" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O210" t="inlineStr">
         <is>
@@ -18141,7 +18141,7 @@
       </c>
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O211" t="inlineStr">
         <is>
@@ -18225,7 +18225,7 @@
       </c>
       <c r="M212" t="inlineStr"/>
       <c r="N212" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O212" t="inlineStr">
         <is>
@@ -18309,7 +18309,7 @@
       </c>
       <c r="M213" t="inlineStr"/>
       <c r="N213" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -18393,7 +18393,7 @@
       </c>
       <c r="M214" t="inlineStr"/>
       <c r="N214" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -18477,7 +18477,7 @@
       </c>
       <c r="M215" t="inlineStr"/>
       <c r="N215" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -18561,7 +18561,7 @@
       </c>
       <c r="M216" t="inlineStr"/>
       <c r="N216" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
@@ -18645,7 +18645,7 @@
       </c>
       <c r="M217" t="inlineStr"/>
       <c r="N217" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -18729,7 +18729,7 @@
       </c>
       <c r="M218" t="inlineStr"/>
       <c r="N218" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -18813,7 +18813,7 @@
       </c>
       <c r="M219" t="inlineStr"/>
       <c r="N219" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O219" t="inlineStr">
         <is>
@@ -18897,7 +18897,7 @@
       </c>
       <c r="M220" t="inlineStr"/>
       <c r="N220" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -18981,7 +18981,7 @@
       </c>
       <c r="M221" t="inlineStr"/>
       <c r="N221" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O221" t="inlineStr">
         <is>
@@ -19065,7 +19065,7 @@
       </c>
       <c r="M222" t="inlineStr"/>
       <c r="N222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O222" t="inlineStr">
         <is>
@@ -19149,7 +19149,7 @@
       </c>
       <c r="M223" t="inlineStr"/>
       <c r="N223" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O223" t="inlineStr">
         <is>
@@ -19233,7 +19233,7 @@
       </c>
       <c r="M224" t="inlineStr"/>
       <c r="N224" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O224" t="inlineStr">
         <is>
@@ -19317,7 +19317,7 @@
       </c>
       <c r="M225" t="inlineStr"/>
       <c r="N225" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -19401,7 +19401,7 @@
       </c>
       <c r="M226" t="inlineStr"/>
       <c r="N226" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -19485,7 +19485,7 @@
       </c>
       <c r="M227" t="inlineStr"/>
       <c r="N227" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -19569,7 +19569,7 @@
       </c>
       <c r="M228" t="inlineStr"/>
       <c r="N228" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -19653,7 +19653,7 @@
       </c>
       <c r="M229" t="inlineStr"/>
       <c r="N229" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O229" t="inlineStr">
         <is>
@@ -19737,7 +19737,7 @@
       </c>
       <c r="M230" t="inlineStr"/>
       <c r="N230" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O230" t="inlineStr">
         <is>
@@ -19821,7 +19821,7 @@
       </c>
       <c r="M231" t="inlineStr"/>
       <c r="N231" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O231" t="inlineStr">
         <is>
@@ -19905,7 +19905,7 @@
       </c>
       <c r="M232" t="inlineStr"/>
       <c r="N232" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O232" t="inlineStr">
         <is>
@@ -19989,7 +19989,7 @@
       </c>
       <c r="M233" t="inlineStr"/>
       <c r="N233" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O233" t="inlineStr">
         <is>
@@ -20073,7 +20073,7 @@
       </c>
       <c r="M234" t="inlineStr"/>
       <c r="N234" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O234" t="inlineStr">
         <is>
@@ -20157,7 +20157,7 @@
       </c>
       <c r="M235" t="inlineStr"/>
       <c r="N235" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O235" t="inlineStr">
         <is>
@@ -20241,7 +20241,7 @@
       </c>
       <c r="M236" t="inlineStr"/>
       <c r="N236" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O236" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="M237" t="inlineStr"/>
       <c r="N237" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -20409,7 +20409,7 @@
       </c>
       <c r="M238" t="inlineStr"/>
       <c r="N238" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -20493,7 +20493,7 @@
       </c>
       <c r="M239" t="inlineStr"/>
       <c r="N239" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O239" t="inlineStr">
         <is>
@@ -20577,7 +20577,7 @@
       </c>
       <c r="M240" t="inlineStr"/>
       <c r="N240" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -20661,7 +20661,7 @@
       </c>
       <c r="M241" t="inlineStr"/>
       <c r="N241" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O241" t="inlineStr">
         <is>
@@ -20745,7 +20745,7 @@
       </c>
       <c r="M242" t="inlineStr"/>
       <c r="N242" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O242" t="inlineStr">
         <is>
@@ -20829,7 +20829,7 @@
       </c>
       <c r="M243" t="inlineStr"/>
       <c r="N243" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
@@ -20913,7 +20913,7 @@
       </c>
       <c r="M244" t="inlineStr"/>
       <c r="N244" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
@@ -20997,7 +20997,7 @@
       </c>
       <c r="M245" t="inlineStr"/>
       <c r="N245" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -21081,7 +21081,7 @@
       </c>
       <c r="M246" t="inlineStr"/>
       <c r="N246" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -21165,7 +21165,7 @@
       </c>
       <c r="M247" t="inlineStr"/>
       <c r="N247" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
@@ -21249,7 +21249,7 @@
       </c>
       <c r="M248" t="inlineStr"/>
       <c r="N248" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -21333,7 +21333,7 @@
       </c>
       <c r="M249" t="inlineStr"/>
       <c r="N249" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
@@ -21417,7 +21417,7 @@
       </c>
       <c r="M250" t="inlineStr"/>
       <c r="N250" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
@@ -21501,7 +21501,7 @@
       </c>
       <c r="M251" t="inlineStr"/>
       <c r="N251" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
@@ -21585,7 +21585,7 @@
       </c>
       <c r="M252" t="inlineStr"/>
       <c r="N252" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -21669,7 +21669,7 @@
       </c>
       <c r="M253" t="inlineStr"/>
       <c r="N253" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -21753,7 +21753,7 @@
       </c>
       <c r="M254" t="inlineStr"/>
       <c r="N254" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
@@ -21837,7 +21837,7 @@
       </c>
       <c r="M255" t="inlineStr"/>
       <c r="N255" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
@@ -21921,7 +21921,7 @@
       </c>
       <c r="M256" t="inlineStr"/>
       <c r="N256" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
@@ -22005,7 +22005,7 @@
       </c>
       <c r="M257" t="inlineStr"/>
       <c r="N257" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
@@ -22089,7 +22089,7 @@
       </c>
       <c r="M258" t="inlineStr"/>
       <c r="N258" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
@@ -22173,7 +22173,7 @@
       </c>
       <c r="M259" t="inlineStr"/>
       <c r="N259" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O259" t="inlineStr">
         <is>
@@ -22257,7 +22257,7 @@
       </c>
       <c r="M260" t="inlineStr"/>
       <c r="N260" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -22341,7 +22341,7 @@
       </c>
       <c r="M261" t="inlineStr"/>
       <c r="N261" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -22425,7 +22425,7 @@
       </c>
       <c r="M262" t="inlineStr"/>
       <c r="N262" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -22509,7 +22509,7 @@
       </c>
       <c r="M263" t="inlineStr"/>
       <c r="N263" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -22593,7 +22593,7 @@
       </c>
       <c r="M264" t="inlineStr"/>
       <c r="N264" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
@@ -22677,7 +22677,7 @@
       </c>
       <c r="M265" t="inlineStr"/>
       <c r="N265" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -22761,7 +22761,7 @@
       </c>
       <c r="M266" t="inlineStr"/>
       <c r="N266" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -22845,7 +22845,7 @@
       </c>
       <c r="M267" t="inlineStr"/>
       <c r="N267" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -22929,7 +22929,7 @@
       </c>
       <c r="M268" t="inlineStr"/>
       <c r="N268" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -23013,7 +23013,7 @@
       </c>
       <c r="M269" t="inlineStr"/>
       <c r="N269" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
@@ -23097,7 +23097,7 @@
       </c>
       <c r="M270" t="inlineStr"/>
       <c r="N270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -23181,7 +23181,7 @@
       </c>
       <c r="M271" t="inlineStr"/>
       <c r="N271" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
@@ -23265,7 +23265,7 @@
       </c>
       <c r="M272" t="inlineStr"/>
       <c r="N272" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -23349,7 +23349,7 @@
       </c>
       <c r="M273" t="inlineStr"/>
       <c r="N273" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
@@ -23433,7 +23433,7 @@
       </c>
       <c r="M274" t="inlineStr"/>
       <c r="N274" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -23517,7 +23517,7 @@
       </c>
       <c r="M275" t="inlineStr"/>
       <c r="N275" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
@@ -23601,7 +23601,7 @@
       </c>
       <c r="M276" t="inlineStr"/>
       <c r="N276" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
@@ -23685,7 +23685,7 @@
       </c>
       <c r="M277" t="inlineStr"/>
       <c r="N277" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -23769,7 +23769,7 @@
       </c>
       <c r="M278" t="inlineStr"/>
       <c r="N278" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -23853,7 +23853,7 @@
       </c>
       <c r="M279" t="inlineStr"/>
       <c r="N279" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -23937,7 +23937,7 @@
       </c>
       <c r="M280" t="inlineStr"/>
       <c r="N280" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
@@ -24021,7 +24021,7 @@
       </c>
       <c r="M281" t="inlineStr"/>
       <c r="N281" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O281" t="inlineStr">
         <is>
@@ -24105,7 +24105,7 @@
       </c>
       <c r="M282" t="inlineStr"/>
       <c r="N282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O282" t="inlineStr">
         <is>
@@ -24189,7 +24189,7 @@
       </c>
       <c r="M283" t="inlineStr"/>
       <c r="N283" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -24273,7 +24273,7 @@
       </c>
       <c r="M284" t="inlineStr"/>
       <c r="N284" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -24357,7 +24357,7 @@
       </c>
       <c r="M285" t="inlineStr"/>
       <c r="N285" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -24441,7 +24441,7 @@
       </c>
       <c r="M286" t="inlineStr"/>
       <c r="N286" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -24525,7 +24525,7 @@
       </c>
       <c r="M287" t="inlineStr"/>
       <c r="N287" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O287" t="inlineStr">
         <is>
@@ -24609,7 +24609,7 @@
       </c>
       <c r="M288" t="inlineStr"/>
       <c r="N288" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -24693,7 +24693,7 @@
       </c>
       <c r="M289" t="inlineStr"/>
       <c r="N289" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O289" t="inlineStr">
         <is>
@@ -24777,7 +24777,7 @@
       </c>
       <c r="M290" t="inlineStr"/>
       <c r="N290" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
@@ -24861,7 +24861,7 @@
       </c>
       <c r="M291" t="inlineStr"/>
       <c r="N291" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O291" t="inlineStr">
         <is>
@@ -24945,7 +24945,7 @@
       </c>
       <c r="M292" t="inlineStr"/>
       <c r="N292" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O292" t="inlineStr">
         <is>
@@ -25029,7 +25029,7 @@
       </c>
       <c r="M293" t="inlineStr"/>
       <c r="N293" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O293" t="inlineStr">
         <is>
@@ -25113,7 +25113,7 @@
       </c>
       <c r="M294" t="inlineStr"/>
       <c r="N294" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O294" t="inlineStr">
         <is>
@@ -25197,7 +25197,7 @@
       </c>
       <c r="M295" t="inlineStr"/>
       <c r="N295" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O295" t="inlineStr">
         <is>
@@ -25281,7 +25281,7 @@
       </c>
       <c r="M296" t="inlineStr"/>
       <c r="N296" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O296" t="inlineStr">
         <is>
@@ -25365,7 +25365,7 @@
       </c>
       <c r="M297" t="inlineStr"/>
       <c r="N297" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O297" t="inlineStr">
         <is>
@@ -25449,7 +25449,7 @@
       </c>
       <c r="M298" t="inlineStr"/>
       <c r="N298" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O298" t="inlineStr">
         <is>
@@ -25533,7 +25533,7 @@
       </c>
       <c r="M299" t="inlineStr"/>
       <c r="N299" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
@@ -25617,7 +25617,7 @@
       </c>
       <c r="M300" t="inlineStr"/>
       <c r="N300" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O300" t="inlineStr">
         <is>
@@ -25701,7 +25701,7 @@
       </c>
       <c r="M301" t="inlineStr"/>
       <c r="N301" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
@@ -25785,7 +25785,7 @@
       </c>
       <c r="M302" t="inlineStr"/>
       <c r="N302" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O302" t="inlineStr">
         <is>
@@ -25869,7 +25869,7 @@
       </c>
       <c r="M303" t="inlineStr"/>
       <c r="N303" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O303" t="inlineStr">
         <is>
@@ -25953,7 +25953,7 @@
       </c>
       <c r="M304" t="inlineStr"/>
       <c r="N304" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O304" t="inlineStr">
         <is>
@@ -26037,7 +26037,7 @@
       </c>
       <c r="M305" t="inlineStr"/>
       <c r="N305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O305" t="inlineStr">
         <is>
@@ -26121,7 +26121,7 @@
       </c>
       <c r="M306" t="inlineStr"/>
       <c r="N306" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O306" t="inlineStr">
         <is>
@@ -26205,7 +26205,7 @@
       </c>
       <c r="M307" t="inlineStr"/>
       <c r="N307" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O307" t="inlineStr">
         <is>
@@ -26289,7 +26289,7 @@
       </c>
       <c r="M308" t="inlineStr"/>
       <c r="N308" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O308" t="inlineStr">
         <is>
@@ -26373,7 +26373,7 @@
       </c>
       <c r="M309" t="inlineStr"/>
       <c r="N309" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O309" t="inlineStr">
         <is>
@@ -26457,7 +26457,7 @@
       </c>
       <c r="M310" t="inlineStr"/>
       <c r="N310" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O310" t="inlineStr">
         <is>
@@ -26541,7 +26541,7 @@
       </c>
       <c r="M311" t="inlineStr"/>
       <c r="N311" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O311" t="inlineStr">
         <is>
@@ -26625,7 +26625,7 @@
       </c>
       <c r="M312" t="inlineStr"/>
       <c r="N312" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O312" t="inlineStr">
         <is>
@@ -26709,7 +26709,7 @@
       </c>
       <c r="M313" t="inlineStr"/>
       <c r="N313" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O313" t="inlineStr">
         <is>
@@ -26793,7 +26793,7 @@
       </c>
       <c r="M314" t="inlineStr"/>
       <c r="N314" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O314" t="inlineStr">
         <is>
@@ -26877,7 +26877,7 @@
       </c>
       <c r="M315" t="inlineStr"/>
       <c r="N315" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O315" t="inlineStr">
         <is>
@@ -26961,7 +26961,7 @@
       </c>
       <c r="M316" t="inlineStr"/>
       <c r="N316" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O316" t="inlineStr">
         <is>
@@ -27045,7 +27045,7 @@
       </c>
       <c r="M317" t="inlineStr"/>
       <c r="N317" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O317" t="inlineStr">
         <is>
@@ -27129,7 +27129,7 @@
       </c>
       <c r="M318" t="inlineStr"/>
       <c r="N318" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O318" t="inlineStr">
         <is>
@@ -27213,7 +27213,7 @@
       </c>
       <c r="M319" t="inlineStr"/>
       <c r="N319" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O319" t="inlineStr">
         <is>
@@ -27297,7 +27297,7 @@
       </c>
       <c r="M320" t="inlineStr"/>
       <c r="N320" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O320" t="inlineStr">
         <is>
@@ -27381,7 +27381,7 @@
       </c>
       <c r="M321" t="inlineStr"/>
       <c r="N321" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O321" t="inlineStr">
         <is>
@@ -27465,7 +27465,7 @@
       </c>
       <c r="M322" t="inlineStr"/>
       <c r="N322" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O322" t="inlineStr">
         <is>
@@ -27549,7 +27549,7 @@
       </c>
       <c r="M323" t="inlineStr"/>
       <c r="N323" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O323" t="inlineStr">
         <is>
@@ -27633,7 +27633,7 @@
       </c>
       <c r="M324" t="inlineStr"/>
       <c r="N324" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O324" t="inlineStr">
         <is>
@@ -27717,7 +27717,7 @@
       </c>
       <c r="M325" t="inlineStr"/>
       <c r="N325" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O325" t="inlineStr">
         <is>
@@ -27801,7 +27801,7 @@
       </c>
       <c r="M326" t="inlineStr"/>
       <c r="N326" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O326" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
       </c>
       <c r="M327" t="inlineStr"/>
       <c r="N327" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O327" t="inlineStr">
         <is>
@@ -27969,7 +27969,7 @@
       </c>
       <c r="M328" t="inlineStr"/>
       <c r="N328" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O328" t="inlineStr">
         <is>
@@ -28053,7 +28053,7 @@
       </c>
       <c r="M329" t="inlineStr"/>
       <c r="N329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O329" t="inlineStr">
         <is>
@@ -28137,7 +28137,7 @@
       </c>
       <c r="M330" t="inlineStr"/>
       <c r="N330" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O330" t="inlineStr">
         <is>
@@ -28221,7 +28221,7 @@
       </c>
       <c r="M331" t="inlineStr"/>
       <c r="N331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O331" t="inlineStr">
         <is>
@@ -28305,7 +28305,7 @@
       </c>
       <c r="M332" t="inlineStr"/>
       <c r="N332" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O332" t="inlineStr">
         <is>
@@ -28389,7 +28389,7 @@
       </c>
       <c r="M333" t="inlineStr"/>
       <c r="N333" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O333" t="inlineStr">
         <is>
@@ -28473,7 +28473,7 @@
       </c>
       <c r="M334" t="inlineStr"/>
       <c r="N334" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O334" t="inlineStr">
         <is>
@@ -28557,7 +28557,7 @@
       </c>
       <c r="M335" t="inlineStr"/>
       <c r="N335" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O335" t="inlineStr">
         <is>
@@ -28641,7 +28641,7 @@
       </c>
       <c r="M336" t="inlineStr"/>
       <c r="N336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O336" t="inlineStr">
         <is>
@@ -28725,7 +28725,7 @@
       </c>
       <c r="M337" t="inlineStr"/>
       <c r="N337" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O337" t="inlineStr">
         <is>
@@ -28809,7 +28809,7 @@
       </c>
       <c r="M338" t="inlineStr"/>
       <c r="N338" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O338" t="inlineStr">
         <is>
@@ -28893,7 +28893,7 @@
       </c>
       <c r="M339" t="inlineStr"/>
       <c r="N339" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O339" t="inlineStr">
         <is>
@@ -28977,7 +28977,7 @@
       </c>
       <c r="M340" t="inlineStr"/>
       <c r="N340" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O340" t="inlineStr">
         <is>
@@ -29061,7 +29061,7 @@
       </c>
       <c r="M341" t="inlineStr"/>
       <c r="N341" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O341" t="inlineStr">
         <is>
@@ -29145,7 +29145,7 @@
       </c>
       <c r="M342" t="inlineStr"/>
       <c r="N342" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O342" t="inlineStr">
         <is>
@@ -29229,7 +29229,7 @@
       </c>
       <c r="M343" t="inlineStr"/>
       <c r="N343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O343" t="inlineStr">
         <is>
@@ -29313,7 +29313,7 @@
       </c>
       <c r="M344" t="inlineStr"/>
       <c r="N344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -29397,7 +29397,7 @@
       </c>
       <c r="M345" t="inlineStr"/>
       <c r="N345" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O345" t="inlineStr">
         <is>
@@ -29481,7 +29481,7 @@
       </c>
       <c r="M346" t="inlineStr"/>
       <c r="N346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O346" t="inlineStr">
         <is>
@@ -29565,7 +29565,7 @@
       </c>
       <c r="M347" t="inlineStr"/>
       <c r="N347" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O347" t="inlineStr">
         <is>
@@ -29649,7 +29649,7 @@
       </c>
       <c r="M348" t="inlineStr"/>
       <c r="N348" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O348" t="inlineStr">
         <is>
@@ -29733,7 +29733,7 @@
       </c>
       <c r="M349" t="inlineStr"/>
       <c r="N349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O349" t="inlineStr">
         <is>
@@ -29817,7 +29817,7 @@
       </c>
       <c r="M350" t="inlineStr"/>
       <c r="N350" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O350" t="inlineStr">
         <is>
@@ -29901,7 +29901,7 @@
       </c>
       <c r="M351" t="inlineStr"/>
       <c r="N351" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O351" t="inlineStr">
         <is>
@@ -29985,7 +29985,7 @@
       </c>
       <c r="M352" t="inlineStr"/>
       <c r="N352" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O352" t="inlineStr">
         <is>
@@ -30069,7 +30069,7 @@
       </c>
       <c r="M353" t="inlineStr"/>
       <c r="N353" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O353" t="inlineStr">
         <is>
@@ -30153,7 +30153,7 @@
       </c>
       <c r="M354" t="inlineStr"/>
       <c r="N354" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O354" t="inlineStr">
         <is>
@@ -30237,7 +30237,7 @@
       </c>
       <c r="M355" t="inlineStr"/>
       <c r="N355" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O355" t="inlineStr">
         <is>
@@ -30321,7 +30321,7 @@
       </c>
       <c r="M356" t="inlineStr"/>
       <c r="N356" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O356" t="inlineStr">
         <is>
@@ -30405,7 +30405,7 @@
       </c>
       <c r="M357" t="inlineStr"/>
       <c r="N357" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O357" t="inlineStr">
         <is>
@@ -30489,7 +30489,7 @@
       </c>
       <c r="M358" t="inlineStr"/>
       <c r="N358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O358" t="inlineStr">
         <is>
@@ -30573,7 +30573,7 @@
       </c>
       <c r="M359" t="inlineStr"/>
       <c r="N359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O359" t="inlineStr">
         <is>
@@ -30657,7 +30657,7 @@
       </c>
       <c r="M360" t="inlineStr"/>
       <c r="N360" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O360" t="inlineStr">
         <is>
@@ -30741,7 +30741,7 @@
       </c>
       <c r="M361" t="inlineStr"/>
       <c r="N361" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O361" t="inlineStr">
         <is>
@@ -30825,7 +30825,7 @@
       </c>
       <c r="M362" t="inlineStr"/>
       <c r="N362" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O362" t="inlineStr">
         <is>
@@ -30909,7 +30909,7 @@
       </c>
       <c r="M363" t="inlineStr"/>
       <c r="N363" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O363" t="inlineStr">
         <is>
@@ -30993,7 +30993,7 @@
       </c>
       <c r="M364" t="inlineStr"/>
       <c r="N364" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O364" t="inlineStr">
         <is>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="M365" t="inlineStr"/>
       <c r="N365" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O365" t="inlineStr">
         <is>
@@ -31161,7 +31161,7 @@
       </c>
       <c r="M366" t="inlineStr"/>
       <c r="N366" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O366" t="inlineStr">
         <is>
@@ -31245,7 +31245,7 @@
       </c>
       <c r="M367" t="inlineStr"/>
       <c r="N367" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O367" t="inlineStr">
         <is>
@@ -31329,7 +31329,7 @@
       </c>
       <c r="M368" t="inlineStr"/>
       <c r="N368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O368" t="inlineStr">
         <is>
@@ -31413,7 +31413,7 @@
       </c>
       <c r="M369" t="inlineStr"/>
       <c r="N369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O369" t="inlineStr">
         <is>
@@ -31497,7 +31497,7 @@
       </c>
       <c r="M370" t="inlineStr"/>
       <c r="N370" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O370" t="inlineStr">
         <is>
@@ -31581,7 +31581,7 @@
       </c>
       <c r="M371" t="inlineStr"/>
       <c r="N371" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O371" t="inlineStr">
         <is>
@@ -31665,7 +31665,7 @@
       </c>
       <c r="M372" t="inlineStr"/>
       <c r="N372" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O372" t="inlineStr">
         <is>
@@ -31749,7 +31749,7 @@
       </c>
       <c r="M373" t="inlineStr"/>
       <c r="N373" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O373" t="inlineStr">
         <is>
@@ -31833,7 +31833,7 @@
       </c>
       <c r="M374" t="inlineStr"/>
       <c r="N374" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O374" t="inlineStr">
         <is>
@@ -31917,7 +31917,7 @@
       </c>
       <c r="M375" t="inlineStr"/>
       <c r="N375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O375" t="inlineStr">
         <is>
@@ -32001,7 +32001,7 @@
       </c>
       <c r="M376" t="inlineStr"/>
       <c r="N376" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O376" t="inlineStr">
         <is>
@@ -32085,7 +32085,7 @@
       </c>
       <c r="M377" t="inlineStr"/>
       <c r="N377" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O377" t="inlineStr">
         <is>
@@ -32169,7 +32169,7 @@
       </c>
       <c r="M378" t="inlineStr"/>
       <c r="N378" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O378" t="inlineStr">
         <is>
@@ -32253,7 +32253,7 @@
       </c>
       <c r="M379" t="inlineStr"/>
       <c r="N379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O379" t="inlineStr">
         <is>
@@ -32337,7 +32337,7 @@
       </c>
       <c r="M380" t="inlineStr"/>
       <c r="N380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O380" t="inlineStr">
         <is>
@@ -32421,7 +32421,7 @@
       </c>
       <c r="M381" t="inlineStr"/>
       <c r="N381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O381" t="inlineStr">
         <is>
@@ -32505,7 +32505,7 @@
       </c>
       <c r="M382" t="inlineStr"/>
       <c r="N382" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O382" t="inlineStr">
         <is>
@@ -32589,7 +32589,7 @@
       </c>
       <c r="M383" t="inlineStr"/>
       <c r="N383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O383" t="inlineStr">
         <is>
@@ -32673,7 +32673,7 @@
       </c>
       <c r="M384" t="inlineStr"/>
       <c r="N384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O384" t="inlineStr">
         <is>
@@ -32757,7 +32757,7 @@
       </c>
       <c r="M385" t="inlineStr"/>
       <c r="N385" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O385" t="inlineStr">
         <is>
@@ -32841,7 +32841,7 @@
       </c>
       <c r="M386" t="inlineStr"/>
       <c r="N386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O386" t="inlineStr">
         <is>
@@ -32925,7 +32925,7 @@
       </c>
       <c r="M387" t="inlineStr"/>
       <c r="N387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O387" t="inlineStr">
         <is>
@@ -33009,7 +33009,7 @@
       </c>
       <c r="M388" t="inlineStr"/>
       <c r="N388" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O388" t="inlineStr">
         <is>
@@ -33093,7 +33093,7 @@
       </c>
       <c r="M389" t="inlineStr"/>
       <c r="N389" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O389" t="inlineStr">
         <is>
@@ -33177,7 +33177,7 @@
       </c>
       <c r="M390" t="inlineStr"/>
       <c r="N390" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O390" t="inlineStr">
         <is>
@@ -33261,7 +33261,7 @@
       </c>
       <c r="M391" t="inlineStr"/>
       <c r="N391" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O391" t="inlineStr">
         <is>
@@ -33345,7 +33345,7 @@
       </c>
       <c r="M392" t="inlineStr"/>
       <c r="N392" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O392" t="inlineStr">
         <is>
@@ -33429,7 +33429,7 @@
       </c>
       <c r="M393" t="inlineStr"/>
       <c r="N393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O393" t="inlineStr">
         <is>
@@ -33513,7 +33513,7 @@
       </c>
       <c r="M394" t="inlineStr"/>
       <c r="N394" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O394" t="inlineStr">
         <is>
@@ -33597,7 +33597,7 @@
       </c>
       <c r="M395" t="inlineStr"/>
       <c r="N395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O395" t="inlineStr">
         <is>
@@ -33681,7 +33681,7 @@
       </c>
       <c r="M396" t="inlineStr"/>
       <c r="N396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O396" t="inlineStr">
         <is>
@@ -33765,7 +33765,7 @@
       </c>
       <c r="M397" t="inlineStr"/>
       <c r="N397" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O397" t="inlineStr">
         <is>
@@ -33849,7 +33849,7 @@
       </c>
       <c r="M398" t="inlineStr"/>
       <c r="N398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O398" t="inlineStr">
         <is>
@@ -33933,7 +33933,7 @@
       </c>
       <c r="M399" t="inlineStr"/>
       <c r="N399" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O399" t="inlineStr">
         <is>
@@ -34017,7 +34017,7 @@
       </c>
       <c r="M400" t="inlineStr"/>
       <c r="N400" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O400" t="inlineStr">
         <is>
@@ -34101,7 +34101,7 @@
       </c>
       <c r="M401" t="inlineStr"/>
       <c r="N401" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O401" t="inlineStr">
         <is>
@@ -34185,7 +34185,7 @@
       </c>
       <c r="M402" t="inlineStr"/>
       <c r="N402" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O402" t="inlineStr">
         <is>
@@ -34269,7 +34269,7 @@
       </c>
       <c r="M403" t="inlineStr"/>
       <c r="N403" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O403" t="inlineStr">
         <is>
@@ -34353,7 +34353,7 @@
       </c>
       <c r="M404" t="inlineStr"/>
       <c r="N404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O404" t="inlineStr">
         <is>
@@ -34437,7 +34437,7 @@
       </c>
       <c r="M405" t="inlineStr"/>
       <c r="N405" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O405" t="inlineStr">
         <is>
@@ -34521,7 +34521,7 @@
       </c>
       <c r="M406" t="inlineStr"/>
       <c r="N406" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O406" t="inlineStr">
         <is>
@@ -34605,7 +34605,7 @@
       </c>
       <c r="M407" t="inlineStr"/>
       <c r="N407" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O407" t="inlineStr">
         <is>
@@ -34689,7 +34689,7 @@
       </c>
       <c r="M408" t="inlineStr"/>
       <c r="N408" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O408" t="inlineStr">
         <is>
@@ -34773,7 +34773,7 @@
       </c>
       <c r="M409" t="inlineStr"/>
       <c r="N409" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O409" t="inlineStr">
         <is>
@@ -34857,7 +34857,7 @@
       </c>
       <c r="M410" t="inlineStr"/>
       <c r="N410" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O410" t="inlineStr">
         <is>
@@ -34941,7 +34941,7 @@
       </c>
       <c r="M411" t="inlineStr"/>
       <c r="N411" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O411" t="inlineStr">
         <is>
@@ -35025,7 +35025,7 @@
       </c>
       <c r="M412" t="inlineStr"/>
       <c r="N412" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O412" t="inlineStr">
         <is>
@@ -35109,7 +35109,7 @@
       </c>
       <c r="M413" t="inlineStr"/>
       <c r="N413" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O413" t="inlineStr">
         <is>
@@ -35193,7 +35193,7 @@
       </c>
       <c r="M414" t="inlineStr"/>
       <c r="N414" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O414" t="inlineStr">
         <is>
@@ -35277,7 +35277,7 @@
       </c>
       <c r="M415" t="inlineStr"/>
       <c r="N415" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O415" t="inlineStr">
         <is>
@@ -35361,7 +35361,7 @@
       </c>
       <c r="M416" t="inlineStr"/>
       <c r="N416" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O416" t="inlineStr">
         <is>
@@ -35445,7 +35445,7 @@
       </c>
       <c r="M417" t="inlineStr"/>
       <c r="N417" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O417" t="inlineStr">
         <is>
@@ -35529,7 +35529,7 @@
       </c>
       <c r="M418" t="inlineStr"/>
       <c r="N418" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O418" t="inlineStr">
         <is>
@@ -35613,7 +35613,7 @@
       </c>
       <c r="M419" t="inlineStr"/>
       <c r="N419" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O419" t="inlineStr">
         <is>
@@ -35697,7 +35697,7 @@
       </c>
       <c r="M420" t="inlineStr"/>
       <c r="N420" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O420" t="inlineStr">
         <is>
@@ -35781,7 +35781,7 @@
       </c>
       <c r="M421" t="inlineStr"/>
       <c r="N421" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O421" t="inlineStr">
         <is>
@@ -35865,7 +35865,7 @@
       </c>
       <c r="M422" t="inlineStr"/>
       <c r="N422" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O422" t="inlineStr">
         <is>
@@ -35949,7 +35949,7 @@
       </c>
       <c r="M423" t="inlineStr"/>
       <c r="N423" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O423" t="inlineStr">
         <is>
@@ -36033,7 +36033,7 @@
       </c>
       <c r="M424" t="inlineStr"/>
       <c r="N424" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O424" t="inlineStr">
         <is>
@@ -36117,7 +36117,7 @@
       </c>
       <c r="M425" t="inlineStr"/>
       <c r="N425" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O425" t="inlineStr">
         <is>
@@ -36201,7 +36201,7 @@
       </c>
       <c r="M426" t="inlineStr"/>
       <c r="N426" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O426" t="inlineStr">
         <is>
@@ -36285,7 +36285,7 @@
       </c>
       <c r="M427" t="inlineStr"/>
       <c r="N427" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O427" t="inlineStr">
         <is>
@@ -36369,7 +36369,7 @@
       </c>
       <c r="M428" t="inlineStr"/>
       <c r="N428" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O428" t="inlineStr">
         <is>
@@ -36453,7 +36453,7 @@
       </c>
       <c r="M429" t="inlineStr"/>
       <c r="N429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O429" t="inlineStr">
         <is>
@@ -36537,7 +36537,7 @@
       </c>
       <c r="M430" t="inlineStr"/>
       <c r="N430" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O430" t="inlineStr">
         <is>
@@ -36621,7 +36621,7 @@
       </c>
       <c r="M431" t="inlineStr"/>
       <c r="N431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O431" t="inlineStr">
         <is>
@@ -36709,7 +36709,7 @@
         </is>
       </c>
       <c r="N432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O432" t="inlineStr">
         <is>
@@ -36724,7 +36724,7 @@
       </c>
       <c r="R432" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:48.747700+00:00</t>
+          <t>2026-05-11T22:05:54.077541+00:00</t>
         </is>
       </c>
     </row>
@@ -36793,7 +36793,7 @@
         </is>
       </c>
       <c r="N433" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O433" t="inlineStr">
         <is>
@@ -36808,7 +36808,7 @@
       </c>
       <c r="R433" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:36.364286+00:00</t>
+          <t>2026-05-11T22:05:54.077541+00:00</t>
         </is>
       </c>
     </row>
@@ -36877,7 +36877,7 @@
         </is>
       </c>
       <c r="N434" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O434" t="inlineStr">
         <is>
@@ -36892,7 +36892,7 @@
       </c>
       <c r="R434" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:50.503843+00:00</t>
+          <t>2026-05-11T22:05:54.077541+00:00</t>
         </is>
       </c>
     </row>
@@ -36961,7 +36961,7 @@
         </is>
       </c>
       <c r="N435" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O435" t="inlineStr">
         <is>
@@ -36976,7 +36976,7 @@
       </c>
       <c r="R435" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:00.077795+00:00</t>
+          <t>2026-05-11T22:05:54.077541+00:00</t>
         </is>
       </c>
     </row>
@@ -37060,7 +37060,7 @@
       </c>
       <c r="R436" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:52.767981+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37144,7 +37144,7 @@
       </c>
       <c r="R437" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:02.337378+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37228,7 +37228,7 @@
       </c>
       <c r="R438" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:38.649869+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37312,7 +37312,7 @@
       </c>
       <c r="R439" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:55.099713+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37396,7 +37396,7 @@
       </c>
       <c r="R440" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:57.533996+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37480,7 +37480,7 @@
       </c>
       <c r="R441" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:04.760520+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37564,7 +37564,7 @@
       </c>
       <c r="R442" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:59.904051+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37648,7 +37648,7 @@
       </c>
       <c r="R443" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:41.043509+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37732,7 +37732,7 @@
       </c>
       <c r="R444" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:07.157955+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37816,7 +37816,7 @@
       </c>
       <c r="R445" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:02.313975+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37900,7 +37900,7 @@
       </c>
       <c r="R446" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:05.039112+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -37984,7 +37984,7 @@
       </c>
       <c r="R447" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:07.333431+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38068,7 +38068,7 @@
       </c>
       <c r="R448" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:09.572980+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38152,7 +38152,7 @@
       </c>
       <c r="R449" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:10.035549+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38236,7 +38236,7 @@
       </c>
       <c r="R450" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:11.912767+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38320,7 +38320,7 @@
       </c>
       <c r="R451" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:11.954217+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38404,7 +38404,7 @@
       </c>
       <c r="R452" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:14.300502+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38488,7 +38488,7 @@
       </c>
       <c r="R453" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:17.053840+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38572,7 +38572,7 @@
       </c>
       <c r="R454" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:43.378048+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38656,7 +38656,7 @@
       </c>
       <c r="R455" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:45.642221+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38740,7 +38740,7 @@
       </c>
       <c r="R456" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:19.310764+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38824,7 +38824,7 @@
       </c>
       <c r="R457" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:14.347784+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38908,7 +38908,7 @@
       </c>
       <c r="R458" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:21.695246+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -38992,7 +38992,7 @@
       </c>
       <c r="R459" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:23.931853+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39076,7 +39076,7 @@
       </c>
       <c r="R460" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:16.729071+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39160,7 +39160,7 @@
       </c>
       <c r="R461" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:47.947838+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39244,7 +39244,7 @@
       </c>
       <c r="R462" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:26.694113+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39328,7 +39328,7 @@
       </c>
       <c r="R463" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:28.937089+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39412,7 +39412,7 @@
       </c>
       <c r="R464" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:50.326816+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39496,7 +39496,7 @@
       </c>
       <c r="R465" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:19.520351+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39580,7 +39580,7 @@
       </c>
       <c r="R466" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:52.743564+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39664,7 +39664,7 @@
       </c>
       <c r="R467" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:21.787082+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39748,7 +39748,7 @@
       </c>
       <c r="R468" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:24.008183+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39832,7 +39832,7 @@
       </c>
       <c r="R469" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:31.171390+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -39916,7 +39916,7 @@
       </c>
       <c r="R470" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:33.517559+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -40000,7 +40000,7 @@
       </c>
       <c r="R471" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:55.487723+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -40084,7 +40084,7 @@
       </c>
       <c r="R472" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:26.359452+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -40168,7 +40168,7 @@
       </c>
       <c r="R473" t="inlineStr">
         <is>
-          <t>2026-05-11T20:33:29.093063+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>
@@ -40252,7 +40252,7 @@
       </c>
       <c r="R474" t="inlineStr">
         <is>
-          <t>2026-05-11T20:32:57.824496+00:00</t>
+          <t>2026-05-12T06:51:32.828510+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model calibration and documentation
</commit_message>
<xml_diff>
--- a/data/tournaments_master.xlsx
+++ b/data/tournaments_master.xlsx
@@ -37021,7 +37021,7 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Подача поздних заявок</t>
+          <t>Все</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
@@ -37060,7 +37060,7 @@
       </c>
       <c r="R436" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37144,7 +37144,7 @@
       </c>
       <c r="R437" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37228,7 +37228,7 @@
       </c>
       <c r="R438" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37312,7 +37312,7 @@
       </c>
       <c r="R439" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37396,7 +37396,7 @@
       </c>
       <c r="R440" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37441,7 +37441,7 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J441" t="inlineStr">
@@ -37480,7 +37480,7 @@
       </c>
       <c r="R441" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37564,7 +37564,7 @@
       </c>
       <c r="R442" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37648,7 +37648,7 @@
       </c>
       <c r="R443" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37732,7 +37732,7 @@
       </c>
       <c r="R444" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37816,7 +37816,7 @@
       </c>
       <c r="R445" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37900,7 +37900,7 @@
       </c>
       <c r="R446" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -37984,7 +37984,7 @@
       </c>
       <c r="R447" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38068,7 +38068,7 @@
       </c>
       <c r="R448" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38152,7 +38152,7 @@
       </c>
       <c r="R449" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38236,7 +38236,7 @@
       </c>
       <c r="R450" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38320,7 +38320,7 @@
       </c>
       <c r="R451" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38404,7 +38404,7 @@
       </c>
       <c r="R452" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38488,7 +38488,7 @@
       </c>
       <c r="R453" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38572,7 +38572,7 @@
       </c>
       <c r="R454" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38656,7 +38656,7 @@
       </c>
       <c r="R455" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38740,7 +38740,7 @@
       </c>
       <c r="R456" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38824,7 +38824,7 @@
       </c>
       <c r="R457" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38908,7 +38908,7 @@
       </c>
       <c r="R458" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -38992,7 +38992,7 @@
       </c>
       <c r="R459" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39076,7 +39076,7 @@
       </c>
       <c r="R460" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39160,7 +39160,7 @@
       </c>
       <c r="R461" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39244,7 +39244,7 @@
       </c>
       <c r="R462" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39328,7 +39328,7 @@
       </c>
       <c r="R463" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39412,7 +39412,7 @@
       </c>
       <c r="R464" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39496,7 +39496,7 @@
       </c>
       <c r="R465" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39580,7 +39580,7 @@
       </c>
       <c r="R466" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39664,7 +39664,7 @@
       </c>
       <c r="R467" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39748,7 +39748,7 @@
       </c>
       <c r="R468" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39832,7 +39832,7 @@
       </c>
       <c r="R469" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -39916,7 +39916,7 @@
       </c>
       <c r="R470" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -40000,7 +40000,7 @@
       </c>
       <c r="R471" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -40084,7 +40084,7 @@
       </c>
       <c r="R472" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -40168,7 +40168,7 @@
       </c>
       <c r="R473" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>
@@ -40252,7 +40252,7 @@
       </c>
       <c r="R474" t="inlineStr">
         <is>
-          <t>2026-05-12T06:51:32.828510+00:00</t>
+          <t>2026-05-14T11:23:51.011172+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh project data and documentation
</commit_message>
<xml_diff>
--- a/data/tournaments_master.xlsx
+++ b/data/tournaments_master.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R474"/>
+  <dimension ref="A1:R502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37021,7 +37021,7 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Все</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
@@ -37045,7 +37045,7 @@
         </is>
       </c>
       <c r="N436" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O436" t="inlineStr">
         <is>
@@ -37060,7 +37060,7 @@
       </c>
       <c r="R436" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37105,7 +37105,7 @@
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>Подача поздних заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
@@ -37129,7 +37129,7 @@
         </is>
       </c>
       <c r="N437" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O437" t="inlineStr">
         <is>
@@ -37144,7 +37144,7 @@
       </c>
       <c r="R437" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37189,7 +37189,7 @@
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>Подача поздних заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
@@ -37213,7 +37213,7 @@
         </is>
       </c>
       <c r="N438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O438" t="inlineStr">
         <is>
@@ -37228,7 +37228,7 @@
       </c>
       <c r="R438" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37273,7 +37273,7 @@
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>Подача поздних заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J439" t="inlineStr">
@@ -37297,7 +37297,7 @@
         </is>
       </c>
       <c r="N439" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O439" t="inlineStr">
         <is>
@@ -37312,7 +37312,7 @@
       </c>
       <c r="R439" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37381,7 +37381,7 @@
         </is>
       </c>
       <c r="N440" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O440" t="inlineStr">
         <is>
@@ -37396,7 +37396,7 @@
       </c>
       <c r="R440" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37465,7 +37465,7 @@
         </is>
       </c>
       <c r="N441" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O441" t="inlineStr">
         <is>
@@ -37480,7 +37480,7 @@
       </c>
       <c r="R441" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37549,7 +37549,7 @@
         </is>
       </c>
       <c r="N442" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O442" t="inlineStr">
         <is>
@@ -37564,7 +37564,7 @@
       </c>
       <c r="R442" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
         </is>
       </c>
       <c r="N443" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O443" t="inlineStr">
         <is>
@@ -37648,7 +37648,7 @@
       </c>
       <c r="R443" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37717,7 +37717,7 @@
         </is>
       </c>
       <c r="N444" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O444" t="inlineStr">
         <is>
@@ -37732,7 +37732,7 @@
       </c>
       <c r="R444" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37801,7 +37801,7 @@
         </is>
       </c>
       <c r="N445" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O445" t="inlineStr">
         <is>
@@ -37816,7 +37816,7 @@
       </c>
       <c r="R445" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-05-17T18:55:42.622398+00:00</t>
         </is>
       </c>
     </row>
@@ -37861,17 +37861,17 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>Подача поздних заявок</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J446" t="inlineStr">
         <is>
-          <t>V А</t>
+          <t>Все</t>
         </is>
       </c>
       <c r="K446" t="inlineStr">
         <is>
-          <t>Олимпийская</t>
+          <t>Все</t>
         </is>
       </c>
       <c r="L446" t="inlineStr">
@@ -37885,14 +37885,18 @@
         </is>
       </c>
       <c r="N446" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O446" t="inlineStr">
         <is>
-          <t>rtt_calendar</t>
-        </is>
-      </c>
-      <c r="P446" t="inlineStr"/>
+          <t>legacy_excel</t>
+        </is>
+      </c>
+      <c r="P446" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q446" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -37900,7 +37904,7 @@
       </c>
       <c r="R446" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:55:30.287435+00:00</t>
         </is>
       </c>
     </row>
@@ -37945,7 +37949,7 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J447" t="inlineStr">
@@ -37969,14 +37973,18 @@
         </is>
       </c>
       <c r="N447" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O447" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P447" t="inlineStr"/>
+      <c r="P447" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q447" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -37984,7 +37992,7 @@
       </c>
       <c r="R447" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:58:31.336903+00:00</t>
         </is>
       </c>
     </row>
@@ -38029,7 +38037,7 @@
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J448" t="inlineStr">
@@ -38053,14 +38061,18 @@
         </is>
       </c>
       <c r="N448" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O448" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P448" t="inlineStr"/>
+      <c r="P448" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q448" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38068,7 +38080,7 @@
       </c>
       <c r="R448" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:58:31.336903+00:00</t>
         </is>
       </c>
     </row>
@@ -38113,7 +38125,7 @@
       </c>
       <c r="I449" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Все</t>
         </is>
       </c>
       <c r="J449" t="inlineStr">
@@ -38137,14 +38149,18 @@
         </is>
       </c>
       <c r="N449" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O449" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P449" t="inlineStr"/>
+      <c r="P449" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q449" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -38152,7 +38168,7 @@
       </c>
       <c r="R449" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:58:31.336903+00:00</t>
         </is>
       </c>
     </row>
@@ -38197,7 +38213,7 @@
       </c>
       <c r="I450" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J450" t="inlineStr">
@@ -38221,14 +38237,18 @@
         </is>
       </c>
       <c r="N450" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O450" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P450" t="inlineStr"/>
+      <c r="P450" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q450" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38236,7 +38256,7 @@
       </c>
       <c r="R450" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:58:31.336903+00:00</t>
         </is>
       </c>
     </row>
@@ -38281,7 +38301,7 @@
       </c>
       <c r="I451" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J451" t="inlineStr">
@@ -38305,14 +38325,18 @@
         </is>
       </c>
       <c r="N451" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O451" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P451" t="inlineStr"/>
+      <c r="P451" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q451" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -38320,7 +38344,7 @@
       </c>
       <c r="R451" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-01T14:58:31.336903+00:00</t>
         </is>
       </c>
     </row>
@@ -38365,7 +38389,7 @@
       </c>
       <c r="I452" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J452" t="inlineStr">
@@ -38389,14 +38413,18 @@
         </is>
       </c>
       <c r="N452" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O452" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P452" t="inlineStr"/>
+      <c r="P452" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q452" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38404,7 +38432,7 @@
       </c>
       <c r="R452" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38449,7 +38477,7 @@
       </c>
       <c r="I453" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J453" t="inlineStr">
@@ -38473,14 +38501,18 @@
         </is>
       </c>
       <c r="N453" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O453" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P453" t="inlineStr"/>
+      <c r="P453" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q453" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38488,7 +38520,7 @@
       </c>
       <c r="R453" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38565,7 @@
       </c>
       <c r="I454" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J454" t="inlineStr">
@@ -38557,14 +38589,18 @@
         </is>
       </c>
       <c r="N454" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O454" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P454" t="inlineStr"/>
+      <c r="P454" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q454" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -38572,7 +38608,7 @@
       </c>
       <c r="R454" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38617,7 +38653,7 @@
       </c>
       <c r="I455" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J455" t="inlineStr">
@@ -38641,14 +38677,18 @@
         </is>
       </c>
       <c r="N455" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O455" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P455" t="inlineStr"/>
+      <c r="P455" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q455" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -38656,7 +38696,7 @@
       </c>
       <c r="R455" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38701,7 +38741,7 @@
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J456" t="inlineStr">
@@ -38725,14 +38765,18 @@
         </is>
       </c>
       <c r="N456" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O456" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P456" t="inlineStr"/>
+      <c r="P456" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q456" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38740,7 +38784,7 @@
       </c>
       <c r="R456" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38785,7 +38829,7 @@
       </c>
       <c r="I457" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J457" t="inlineStr">
@@ -38809,14 +38853,18 @@
         </is>
       </c>
       <c r="N457" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O457" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P457" t="inlineStr"/>
+      <c r="P457" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q457" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -38824,7 +38872,7 @@
       </c>
       <c r="R457" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38869,7 +38917,7 @@
       </c>
       <c r="I458" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J458" t="inlineStr">
@@ -38893,14 +38941,18 @@
         </is>
       </c>
       <c r="N458" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O458" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P458" t="inlineStr"/>
+      <c r="P458" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q458" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38908,7 +38960,7 @@
       </c>
       <c r="R458" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -38953,7 +39005,7 @@
       </c>
       <c r="I459" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J459" t="inlineStr">
@@ -38977,14 +39029,18 @@
         </is>
       </c>
       <c r="N459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O459" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P459" t="inlineStr"/>
+      <c r="P459" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q459" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -38992,7 +39048,7 @@
       </c>
       <c r="R459" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -39037,7 +39093,7 @@
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J460" t="inlineStr">
@@ -39061,14 +39117,18 @@
         </is>
       </c>
       <c r="N460" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O460" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P460" t="inlineStr"/>
+      <c r="P460" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q460" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -39076,7 +39136,7 @@
       </c>
       <c r="R460" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -39121,7 +39181,7 @@
       </c>
       <c r="I461" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J461" t="inlineStr">
@@ -39145,14 +39205,18 @@
         </is>
       </c>
       <c r="N461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O461" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P461" t="inlineStr"/>
+      <c r="P461" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q461" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -39160,7 +39224,7 @@
       </c>
       <c r="R461" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -39205,7 +39269,7 @@
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J462" t="inlineStr">
@@ -39229,14 +39293,18 @@
         </is>
       </c>
       <c r="N462" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O462" t="inlineStr">
         <is>
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P462" t="inlineStr"/>
+      <c r="P462" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q462" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -39244,7 +39312,7 @@
       </c>
       <c r="R462" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-08T06:20:27.286668+00:00</t>
         </is>
       </c>
     </row>
@@ -39289,7 +39357,7 @@
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J463" t="inlineStr">
@@ -39320,7 +39388,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P463" t="inlineStr"/>
+      <c r="P463" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q463" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -39328,7 +39400,7 @@
       </c>
       <c r="R463" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
@@ -39373,7 +39445,7 @@
       </c>
       <c r="I464" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>В процессе проведения</t>
         </is>
       </c>
       <c r="J464" t="inlineStr">
@@ -39404,7 +39476,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P464" t="inlineStr"/>
+      <c r="P464" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q464" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -39412,7 +39488,7 @@
       </c>
       <c r="R464" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
@@ -39457,7 +39533,7 @@
       </c>
       <c r="I465" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J465" t="inlineStr">
@@ -39488,7 +39564,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P465" t="inlineStr"/>
+      <c r="P465" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q465" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -39496,7 +39576,7 @@
       </c>
       <c r="R465" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
@@ -39541,7 +39621,7 @@
       </c>
       <c r="I466" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J466" t="inlineStr">
@@ -39572,7 +39652,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P466" t="inlineStr"/>
+      <c r="P466" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q466" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -39580,7 +39664,7 @@
       </c>
       <c r="R466" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
@@ -39625,7 +39709,7 @@
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J467" t="inlineStr">
@@ -39656,7 +39740,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P467" t="inlineStr"/>
+      <c r="P467" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q467" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -39664,7 +39752,7 @@
       </c>
       <c r="R467" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
@@ -39709,7 +39797,7 @@
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J468" t="inlineStr">
@@ -39740,7 +39828,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P468" t="inlineStr"/>
+      <c r="P468" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q468" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:44.681774+00:00</t>
@@ -39748,24 +39840,24 @@
       </c>
       <c r="R468" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>305454</t>
+          <t>305659</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>Первенство Рязанской области</t>
+          <t>Чемпионат и Первенство Сергиево-Посадского городского округа "Золотые Купола"</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>до 17 лет</t>
+          <t>Взрослые</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -39785,20 +39877,20 @@
       </c>
       <c r="G469" t="inlineStr">
         <is>
-          <t>Рязань</t>
+          <t>Сергиев Посад</t>
         </is>
       </c>
       <c r="H469" s="2" t="n">
-        <v>46202</v>
+        <v>46195</v>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J469" t="inlineStr">
         <is>
-          <t>III А</t>
+          <t>IV А</t>
         </is>
       </c>
       <c r="K469" t="inlineStr">
@@ -39808,12 +39900,12 @@
       </c>
       <c r="L469" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305454/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305659/matches</t>
         </is>
       </c>
       <c r="M469" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305454/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305659/dashboard</t>
         </is>
       </c>
       <c r="N469" t="b">
@@ -39824,27 +39916,31 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P469" t="inlineStr"/>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q469" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:12.363735+00:00</t>
+          <t>2026-05-29T06:02:24.670683+00:00</t>
         </is>
       </c>
       <c r="R469" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>305217</t>
+          <t>305454</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Турнир Кубок "Мостеннис"</t>
+          <t>Первенство Рязанской области</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -39869,20 +39965,20 @@
       </c>
       <c r="G470" t="inlineStr">
         <is>
-          <t>Воскресенск</t>
+          <t>Рязань</t>
         </is>
       </c>
       <c r="H470" s="2" t="n">
-        <v>46207</v>
+        <v>46202</v>
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J470" t="inlineStr">
         <is>
-          <t>V А</t>
+          <t>III А</t>
         </is>
       </c>
       <c r="K470" t="inlineStr">
@@ -39892,12 +39988,12 @@
       </c>
       <c r="L470" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305217/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305454/matches</t>
         </is>
       </c>
       <c r="M470" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305217/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305454/dashboard</t>
         </is>
       </c>
       <c r="N470" t="b">
@@ -39908,7 +40004,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P470" t="inlineStr"/>
+      <c r="P470" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q470" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:12.363735+00:00</t>
@@ -39916,24 +40016,24 @@
       </c>
       <c r="R470" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>305559</t>
+          <t>305692</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>Кубок Федерации тенниса Воронежской области</t>
+          <t>Турнир "Кубок Жемчужины Подмосковья"</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>до 19 лет</t>
+          <t>до 17 лет</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -39953,20 +40053,20 @@
       </c>
       <c r="G471" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>Истра</t>
         </is>
       </c>
       <c r="H471" s="2" t="n">
-        <v>46209</v>
+        <v>46202</v>
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J471" t="inlineStr">
         <is>
-          <t>III Б</t>
+          <t>IV Б</t>
         </is>
       </c>
       <c r="K471" t="inlineStr">
@@ -39976,12 +40076,12 @@
       </c>
       <c r="L471" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305559/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305692/matches</t>
         </is>
       </c>
       <c r="M471" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305559/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305692/dashboard</t>
         </is>
       </c>
       <c r="N471" t="b">
@@ -39992,32 +40092,36 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P471" t="inlineStr"/>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q471" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:28.549184+00:00</t>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
         </is>
       </c>
       <c r="R471" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>305505</t>
+          <t>305757</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>Турнир города Москвы А Л Т - ИЮЛЬ (Включен в ЕКП Москомспорта)</t>
+          <t>Первенство Одинцовского городского округа Московской области "Гранд Теннис"</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>Взрослые</t>
+          <t>до 17 лет</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -40037,20 +40141,20 @@
       </c>
       <c r="G472" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Одинцово</t>
         </is>
       </c>
       <c r="H472" s="2" t="n">
-        <v>46216</v>
+        <v>46202</v>
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J472" t="inlineStr">
         <is>
-          <t>V Б</t>
+          <t>IV А</t>
         </is>
       </c>
       <c r="K472" t="inlineStr">
@@ -40060,12 +40164,12 @@
       </c>
       <c r="L472" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305505/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305757/matches</t>
         </is>
       </c>
       <c r="M472" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305505/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305757/dashboard</t>
         </is>
       </c>
       <c r="N472" t="b">
@@ -40076,27 +40180,31 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P472" t="inlineStr"/>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q472" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:44.681774+00:00</t>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
         </is>
       </c>
       <c r="R472" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>305578</t>
+          <t>305769</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>Всероссийские соревнования</t>
+          <t>Чемпионат Одинцовского городского округа Московской области "Гранд Теннис"</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
@@ -40121,20 +40229,20 @@
       </c>
       <c r="G473" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Одинцово</t>
         </is>
       </c>
       <c r="H473" s="2" t="n">
-        <v>46223</v>
+        <v>46202</v>
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>Подача заявок</t>
+          <t>Подача поздних заявок</t>
         </is>
       </c>
       <c r="J473" t="inlineStr">
         <is>
-          <t>I А</t>
+          <t>IV А</t>
         </is>
       </c>
       <c r="K473" t="inlineStr">
@@ -40144,12 +40252,12 @@
       </c>
       <c r="L473" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305578/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305769/matches</t>
         </is>
       </c>
       <c r="M473" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305578/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305769/dashboard</t>
         </is>
       </c>
       <c r="N473" t="b">
@@ -40160,27 +40268,31 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P473" t="inlineStr"/>
+      <c r="P473" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q473" t="inlineStr">
         <is>
-          <t>2026-05-11T20:31:44.681774+00:00</t>
+          <t>2026-05-29T06:02:24.670683+00:00</t>
         </is>
       </c>
       <c r="R473" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>305529</t>
+          <t>305559</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>Первенство Тверской области</t>
+          <t>Кубок Федерации тенниса Воронежской области</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -40205,11 +40317,11 @@
       </c>
       <c r="G474" t="inlineStr">
         <is>
-          <t>Вышний Волочек</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="H474" s="2" t="n">
-        <v>46230</v>
+        <v>46209</v>
       </c>
       <c r="I474" t="inlineStr">
         <is>
@@ -40218,22 +40330,22 @@
       </c>
       <c r="J474" t="inlineStr">
         <is>
-          <t>III А</t>
+          <t>III Б</t>
         </is>
       </c>
       <c r="K474" t="inlineStr">
         <is>
-          <t>Олимпийская</t>
+          <t>Олимпийская и ДТ</t>
         </is>
       </c>
       <c r="L474" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305529/matches</t>
+          <t>https://rtt.mytennis.online/public/tours/305559/matches</t>
         </is>
       </c>
       <c r="M474" t="inlineStr">
         <is>
-          <t>https://rtt.mytennis.online/public/tours/305529/dashboard</t>
+          <t>https://rtt.mytennis.online/public/tours/305559/dashboard</t>
         </is>
       </c>
       <c r="N474" t="b">
@@ -40244,7 +40356,11 @@
           <t>rtt_calendar</t>
         </is>
       </c>
-      <c r="P474" t="inlineStr"/>
+      <c r="P474" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
       <c r="Q474" t="inlineStr">
         <is>
           <t>2026-05-11T20:31:28.549184+00:00</t>
@@ -40252,7 +40368,2415 @@
       </c>
       <c r="R474" t="inlineStr">
         <is>
-          <t>2026-05-14T11:23:51.011172+00:00</t>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>305907</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Чемпионат и Первенство Сергиево-Посадского городского округа "Золотые Купола"</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>Сергиев Посад</t>
+        </is>
+      </c>
+      <c r="H475" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305907/matches</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305907/dashboard</t>
+        </is>
+      </c>
+      <c r="N475" t="b">
+        <v>0</v>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P475" t="inlineStr"/>
+      <c r="Q475" t="inlineStr">
+        <is>
+          <t>2026-06-01T14:56:41.903320+00:00</t>
+        </is>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>305908</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Чемпионат и Первенство Сергиево-Посадского городского округа "Золотые Купола"</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>Сергиев Посад</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305908/matches</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305908/dashboard</t>
+        </is>
+      </c>
+      <c r="N476" t="b">
+        <v>0</v>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P476" t="inlineStr"/>
+      <c r="Q476" t="inlineStr">
+        <is>
+          <t>2026-06-01T14:56:07.658244+00:00</t>
+        </is>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>305963</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Первенство г. Люберцы "Люберцы ОПЕН"</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>до 19 лет</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Люберцы</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305963/matches</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305963/dashboard</t>
+        </is>
+      </c>
+      <c r="N477" t="b">
+        <v>0</v>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P477" t="inlineStr"/>
+      <c r="Q477" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:56.629283+00:00</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>305217</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Турнир Кубок "Мостеннис"</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Воскресенск</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>V А</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305217/matches</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305217/dashboard</t>
+        </is>
+      </c>
+      <c r="N478" t="b">
+        <v>0</v>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P478" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q478" t="inlineStr">
+        <is>
+          <t>2026-05-11T20:31:12.363735+00:00</t>
+        </is>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>305505</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Турнир города Москвы А Л Т - ИЮЛЬ (Включен в ЕКП Москомспорта)</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>V Б</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305505/matches</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305505/dashboard</t>
+        </is>
+      </c>
+      <c r="N479" t="b">
+        <v>0</v>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P479" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q479" t="inlineStr">
+        <is>
+          <t>2026-05-11T20:31:44.681774+00:00</t>
+        </is>
+      </c>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>305652</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Областные Соревнования "Турнир на призы Федерации тенниса Тульской области"</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Тула</t>
+        </is>
+      </c>
+      <c r="H480" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>III А</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305652/matches</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305652/dashboard</t>
+        </is>
+      </c>
+      <c r="N480" t="b">
+        <v>0</v>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P480" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q480" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>305668</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Первенство городского округа Воскресенск на призы TENNIS LIFE</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Воскресенск</t>
+        </is>
+      </c>
+      <c r="H481" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305668/matches</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305668/dashboard</t>
+        </is>
+      </c>
+      <c r="N481" t="b">
+        <v>0</v>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P481" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q481" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>305729</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Турнир, посвященный памяти О. Л. Корнблита</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="H482" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>IV Б</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305729/matches</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305729/dashboard</t>
+        </is>
+      </c>
+      <c r="N482" t="b">
+        <v>0</v>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P482" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>305932</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Первенство Центрального Федерального округа</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Калуга</t>
+        </is>
+      </c>
+      <c r="H483" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>I Б</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305932/matches</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305932/dashboard</t>
+        </is>
+      </c>
+      <c r="N483" t="b">
+        <v>0</v>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P483" t="inlineStr"/>
+      <c r="Q483" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>306008</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Чемпионат Одинцовского городского округа Московской области "Гранд Теннис"</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>Одинцово</t>
+        </is>
+      </c>
+      <c r="H484" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306008/matches</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306008/dashboard</t>
+        </is>
+      </c>
+      <c r="N484" t="b">
+        <v>0</v>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P484" t="inlineStr"/>
+      <c r="Q484" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:18:13.756561+00:00</t>
+        </is>
+      </c>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>305578</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Всероссийские соревнования</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="H485" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>I А</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305578/matches</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305578/dashboard</t>
+        </is>
+      </c>
+      <c r="N485" t="b">
+        <v>0</v>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P485" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q485" t="inlineStr">
+        <is>
+          <t>2026-05-11T20:31:44.681774+00:00</t>
+        </is>
+      </c>
+      <c r="R485" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>305813</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Кубок Липецкой области Федерации тенниса</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>Липецк</t>
+        </is>
+      </c>
+      <c r="H486" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>III Б</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305813/matches</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305813/dashboard</t>
+        </is>
+      </c>
+      <c r="N486" t="b">
+        <v>0</v>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P486" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q486" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>305883</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Первенство Курской области</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>Курск</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>III А</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305883/matches</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305883/dashboard</t>
+        </is>
+      </c>
+      <c r="N487" t="b">
+        <v>0</v>
+      </c>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P487" t="inlineStr"/>
+      <c r="Q487" t="inlineStr">
+        <is>
+          <t>2026-05-31T07:08:16.640326+00:00</t>
+        </is>
+      </c>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>305529</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Первенство Тверской области</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>до 19 лет</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Вышний Волочек</t>
+        </is>
+      </c>
+      <c r="H488" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>III А</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305529/matches</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305529/dashboard</t>
+        </is>
+      </c>
+      <c r="N488" t="b">
+        <v>0</v>
+      </c>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P488" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q488" t="inlineStr">
+        <is>
+          <t>2026-05-11T20:31:28.549184+00:00</t>
+        </is>
+      </c>
+      <c r="R488" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>305761</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>"Рязанская ракетка"</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>IV Б</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305761/matches</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305761/dashboard</t>
+        </is>
+      </c>
+      <c r="N489" t="b">
+        <v>0</v>
+      </c>
+      <c r="O489" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P489" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q489" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R489" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>306021</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Первенство Одинцовского городского округа Московской области "Гранд Теннис"</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>Одинцово</t>
+        </is>
+      </c>
+      <c r="H490" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306021/matches</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306021/dashboard</t>
+        </is>
+      </c>
+      <c r="N490" t="b">
+        <v>0</v>
+      </c>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P490" t="inlineStr"/>
+      <c r="Q490" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R490" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>306026</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Чемпионат Одинцовского городского округа Московской области "Гранд Теннис"</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>Одинцово</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306026/matches</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306026/dashboard</t>
+        </is>
+      </c>
+      <c r="N491" t="b">
+        <v>0</v>
+      </c>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P491" t="inlineStr"/>
+      <c r="Q491" t="inlineStr">
+        <is>
+          <t>2026-06-19T18:20:06.082069+00:00</t>
+        </is>
+      </c>
+      <c r="R491" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>305988</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Кубок Федерации тенниса Рязанской области</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="H492" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>III Б</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305988/matches</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305988/dashboard</t>
+        </is>
+      </c>
+      <c r="N492" t="b">
+        <v>0</v>
+      </c>
+      <c r="O492" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P492" t="inlineStr"/>
+      <c r="Q492" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:18:13.756561+00:00</t>
+        </is>
+      </c>
+      <c r="R492" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>305991</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Кубок Федерации тенниса Рязанской области</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>Рязань</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>III Б</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305991/matches</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305991/dashboard</t>
+        </is>
+      </c>
+      <c r="N493" t="b">
+        <v>0</v>
+      </c>
+      <c r="O493" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P493" t="inlineStr"/>
+      <c r="Q493" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R493" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>306032</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>ЛЕТНИЙ ЧЕМПИОНАТ МОСКВЫ</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="H494" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>МТ ФТР</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306032/matches</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306032/dashboard</t>
+        </is>
+      </c>
+      <c r="N494" t="b">
+        <v>0</v>
+      </c>
+      <c r="O494" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P494" t="inlineStr"/>
+      <c r="Q494" t="inlineStr">
+        <is>
+          <t>2026-06-19T18:20:06.082069+00:00</t>
+        </is>
+      </c>
+      <c r="R494" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>305772</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Турнир Кубок "Мостеннис"</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>Воскресенск</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>V А</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305772/matches</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305772/dashboard</t>
+        </is>
+      </c>
+      <c r="N495" t="b">
+        <v>0</v>
+      </c>
+      <c r="O495" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P495" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q495" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R495" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>306006</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Турнир выходного дня "Золотые Купола"</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>Сергиев Посад</t>
+        </is>
+      </c>
+      <c r="H496" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>V А</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306006/matches</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/306006/dashboard</t>
+        </is>
+      </c>
+      <c r="N496" t="b">
+        <v>0</v>
+      </c>
+      <c r="O496" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P496" t="inlineStr"/>
+      <c r="Q496" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R496" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>305618</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Турнир А Л Т - Август (Включен в ЕКП Москомспорта)</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>V Б</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305618/matches</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305618/dashboard</t>
+        </is>
+      </c>
+      <c r="N497" t="b">
+        <v>0</v>
+      </c>
+      <c r="O497" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P497" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q497" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>305784</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Первенство городского округа Воскресенск на призы TENNIS LIFE</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>Воскресенск</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>IV А</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305784/matches</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305784/dashboard</t>
+        </is>
+      </c>
+      <c r="N498" t="b">
+        <v>0</v>
+      </c>
+      <c r="O498" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P498" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q498" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R498" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>305873</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Всероссийские соревнования</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Взрослые</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>I А</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>Олимпийская и ДТ</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305873/matches</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305873/dashboard</t>
+        </is>
+      </c>
+      <c r="N499" t="b">
+        <v>0</v>
+      </c>
+      <c r="O499" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P499" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q499" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:02:24.670683+00:00</t>
+        </is>
+      </c>
+      <c r="R499" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>305918</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Кубок Федерации тенниса Липецкой области</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>Липецк</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>III Б</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305918/matches</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305918/dashboard</t>
+        </is>
+      </c>
+      <c r="N500" t="b">
+        <v>0</v>
+      </c>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P500" t="inlineStr"/>
+      <c r="Q500" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R500" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>305978</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Турнир Кубок "Мостеннис"</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>Дмитров</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>V А</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305978/matches</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305978/dashboard</t>
+        </is>
+      </c>
+      <c r="N501" t="b">
+        <v>0</v>
+      </c>
+      <c r="O501" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P501" t="inlineStr"/>
+      <c r="Q501" t="inlineStr">
+        <is>
+          <t>2026-06-08T06:17:39.386698+00:00</t>
+        </is>
+      </c>
+      <c r="R501" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>305791</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Турнир Кубок "Мостеннис"</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>до 17 лет</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Женский</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Одиночный</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Центральный ФО</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>Воскресенск</t>
+        </is>
+      </c>
+      <c r="H502" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Подача заявок</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>V А</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>Олимпийская</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305791/matches</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>https://rtt.mytennis.online/public/tours/305791/dashboard</t>
+        </is>
+      </c>
+      <c r="N502" t="b">
+        <v>0</v>
+      </c>
+      <c r="O502" t="inlineStr">
+        <is>
+          <t>rtt_calendar</t>
+        </is>
+      </c>
+      <c r="P502" t="inlineStr">
+        <is>
+          <t>rtt_failed_links.xlsx</t>
+        </is>
+      </c>
+      <c r="Q502" t="inlineStr">
+        <is>
+          <t>2026-05-29T06:01:50.436836+00:00</t>
+        </is>
+      </c>
+      <c r="R502" t="inlineStr">
+        <is>
+          <t>2026-06-19T20:45:21.057124+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>